<commit_message>
Commit from thinkpad on 12/05/2026, 15:14:08
</commit_message>
<xml_diff>
--- a/Entregas PhD/EntregaResearch.xlsx
+++ b/Entregas PhD/EntregaResearch.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/rdpds/Documents/Obsidian/phd-vault/Entregas PhD/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{89A3DA10-2310-B94F-8CFF-6262E69033DB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{14667670-8E47-6F49-BA49-6D90B66EDA80}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="600" windowWidth="38400" windowHeight="19320" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -835,6 +835,9 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <sheetPr>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
   <dimension ref="A1:O34"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
@@ -1695,5 +1698,6 @@
     <hyperlink ref="D34" r:id="rId12" xr:uid="{E2A89752-8ED9-5445-B2ED-AAD89618E041}"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup paperSize="9" scale="37" orientation="landscape" horizontalDpi="0" verticalDpi="0"/>
 </worksheet>
 </file>
</xml_diff>